<commit_message>
feat: finish up excel file
</commit_message>
<xml_diff>
--- a/final-project/uthai2.xlsx
+++ b/final-project/uthai2.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="อำเภอบ้านไร่" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="อำเภอลานสัก" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="อำเภอหนองฉาง" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="อำเภอห้วยคต" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="อำเภอบ้านไร่" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="อำเภอลานสัก" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="อำเภอหนองฉาง" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="อำเภอห้วยคต" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>ล่วงหน้านอกเขตและนอกราชอาณาจักร</t>
@@ -501,7 +500,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>ล่วงหน้าในเขต</t>
@@ -553,6 +551,11 @@
           <t>ตำบลคอกควาย</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -560,6 +563,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -567,6 +575,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -574,6 +587,11 @@
       </c>
     </row>
     <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -581,6 +599,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 5 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -588,6 +611,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -595,6 +623,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 7 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -602,6 +635,11 @@
       </c>
     </row>
     <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 8 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -609,6 +647,11 @@
       </c>
     </row>
     <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 9 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -616,6 +659,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 10 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -623,6 +671,11 @@
       </c>
     </row>
     <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 11 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -630,6 +683,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 12 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -637,6 +695,11 @@
       </c>
     </row>
     <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 13 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -644,6 +707,11 @@
       </c>
     </row>
     <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 14 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -651,6 +719,11 @@
       </c>
     </row>
     <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 15 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -658,6 +731,11 @@
       </c>
     </row>
     <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 16 ตำบลคอกควาย</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>หน่วย 16</t>
@@ -670,6 +748,11 @@
           <t>ตำบลทัพหลวง</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 1 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -677,6 +760,11 @@
       </c>
     </row>
     <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -684,6 +772,11 @@
       </c>
     </row>
     <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -691,6 +784,11 @@
       </c>
     </row>
     <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 4 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -698,6 +796,11 @@
       </c>
     </row>
     <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 5 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -705,6 +808,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -712,6 +820,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 7 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -719,6 +832,11 @@
       </c>
     </row>
     <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 8 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -726,6 +844,11 @@
       </c>
     </row>
     <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 9 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -733,6 +856,11 @@
       </c>
     </row>
     <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 10 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -740,6 +868,11 @@
       </c>
     </row>
     <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 11 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -747,6 +880,11 @@
       </c>
     </row>
     <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 12 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -754,6 +892,11 @@
       </c>
     </row>
     <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 13 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -761,6 +904,11 @@
       </c>
     </row>
     <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 14 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -768,6 +916,11 @@
       </c>
     </row>
     <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 15 ตำบลทัพหลวง</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -780,6 +933,11 @@
           <t>ตำบลบ้านบึง</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -787,6 +945,11 @@
       </c>
     </row>
     <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 2 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -794,6 +957,11 @@
       </c>
     </row>
     <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 3 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -801,6 +969,11 @@
       </c>
     </row>
     <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -808,6 +981,11 @@
       </c>
     </row>
     <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 5 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -815,6 +993,11 @@
       </c>
     </row>
     <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>โรงเรียนวังตอสามัคคี  หมู่ที่ 6 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -822,6 +1005,11 @@
       </c>
     </row>
     <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 7 ตำบลบ้านบึง</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -834,6 +1022,11 @@
           <t>ตำบลบ้านใหม่คลองเคียน</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C40" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -841,6 +1034,11 @@
       </c>
     </row>
     <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 2 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C41" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -848,6 +1046,11 @@
       </c>
     </row>
     <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C42" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -855,6 +1058,11 @@
       </c>
     </row>
     <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C43" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -862,6 +1070,11 @@
       </c>
     </row>
     <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 5 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C44" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -869,6 +1082,11 @@
       </c>
     </row>
     <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -876,6 +1094,11 @@
       </c>
     </row>
     <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 7 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -883,6 +1106,11 @@
       </c>
     </row>
     <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 8 ตำบลบ้านใหม่คลองเคียน</t>
+        </is>
+      </c>
       <c r="C47" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -895,6 +1123,11 @@
           <t>ตำบลบ้านไร่</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C48" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -902,6 +1135,11 @@
       </c>
     </row>
     <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>อาคารกองทุนหมู่บ้าน  หมู่ที่ 2 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C49" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -909,6 +1147,11 @@
       </c>
     </row>
     <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C50" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -916,6 +1159,11 @@
       </c>
     </row>
     <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 4 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C51" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -923,6 +1171,11 @@
       </c>
     </row>
     <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 5 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C52" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -930,6 +1183,11 @@
       </c>
     </row>
     <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 6 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -937,6 +1195,11 @@
       </c>
     </row>
     <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านห้วยป่าปก  หมู่ที่ 7 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -944,6 +1207,11 @@
       </c>
     </row>
     <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 8 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C55" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -951,6 +1219,11 @@
       </c>
     </row>
     <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 9 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C56" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -958,6 +1231,11 @@
       </c>
     </row>
     <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 10 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C57" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -965,6 +1243,11 @@
       </c>
     </row>
     <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 11 ตำบลบ้านไร่</t>
+        </is>
+      </c>
       <c r="C58" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -977,6 +1260,11 @@
           <t>ตำบลวังหิน</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลวังหิน</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -984,6 +1272,11 @@
       </c>
     </row>
     <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลวังหิน</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -991,6 +1284,11 @@
       </c>
     </row>
     <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 3 ตำบลวังหิน</t>
+        </is>
+      </c>
       <c r="C61" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -998,6 +1296,11 @@
       </c>
     </row>
     <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 4 ตำบลวังหิน</t>
+        </is>
+      </c>
       <c r="C62" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1005,6 +1308,11 @@
       </c>
     </row>
     <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 5 ตำบลวังหิน</t>
+        </is>
+      </c>
       <c r="C63" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1012,6 +1320,11 @@
       </c>
     </row>
     <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลวังหิน</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1024,6 +1337,11 @@
           <t>ตำบลหนองจอก</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C65" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1031,6 +1349,11 @@
       </c>
     </row>
     <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 2 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1038,6 +1361,11 @@
       </c>
     </row>
     <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่  3  ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1045,6 +1373,11 @@
       </c>
     </row>
     <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C68" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1052,6 +1385,11 @@
       </c>
     </row>
     <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 5 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C69" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1059,6 +1397,11 @@
       </c>
     </row>
     <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C70" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1066,6 +1409,11 @@
       </c>
     </row>
     <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 7 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C71" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1073,6 +1421,11 @@
       </c>
     </row>
     <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 8 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C72" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1080,6 +1433,11 @@
       </c>
     </row>
     <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน    หมู่ที่ 9 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C73" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1087,6 +1445,11 @@
       </c>
     </row>
     <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 10 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C74" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1094,6 +1457,11 @@
       </c>
     </row>
     <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 11 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C75" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1101,6 +1469,11 @@
       </c>
     </row>
     <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 12 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C76" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -1108,6 +1481,11 @@
       </c>
     </row>
     <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 13 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C77" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -1115,6 +1493,11 @@
       </c>
     </row>
     <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 14 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C78" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -1122,6 +1505,11 @@
       </c>
     </row>
     <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 15 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C79" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -1129,6 +1517,11 @@
       </c>
     </row>
     <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 16 ตำบลหนองจอก</t>
+        </is>
+      </c>
       <c r="C80" t="inlineStr">
         <is>
           <t>หน่วย 16</t>
@@ -1141,6 +1534,11 @@
           <t>ตำบลหนองบ่มกล้วย</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C81" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1148,6 +1546,11 @@
       </c>
     </row>
     <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ศาลาศูนย์ทอผ้าบ้านทุ่งนาสวน  หมู่ที่ 2 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C82" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1155,6 +1558,11 @@
       </c>
     </row>
     <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C83" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1162,6 +1570,11 @@
       </c>
     </row>
     <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C84" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1169,6 +1582,11 @@
       </c>
     </row>
     <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 5 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C85" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1176,6 +1594,11 @@
       </c>
     </row>
     <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 6 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C86" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1183,6 +1606,11 @@
       </c>
     </row>
     <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 7 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C87" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1190,6 +1618,11 @@
       </c>
     </row>
     <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 8 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1197,6 +1630,11 @@
       </c>
     </row>
     <row r="89">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 9 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C89" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1204,6 +1642,11 @@
       </c>
     </row>
     <row r="90">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 10 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C90" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1211,6 +1654,11 @@
       </c>
     </row>
     <row r="91">
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 11 ตำบลหนองบ่มกล้วย</t>
+        </is>
+      </c>
       <c r="C91" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1223,6 +1671,11 @@
           <t>ตำบลหูช้าง</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C92" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1230,6 +1683,11 @@
       </c>
     </row>
     <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C93" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1237,6 +1695,11 @@
       </c>
     </row>
     <row r="94">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน หมู่ที่ 3 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C94" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1244,6 +1707,11 @@
       </c>
     </row>
     <row r="95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C95" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1251,6 +1719,11 @@
       </c>
     </row>
     <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 5 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C96" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1258,6 +1731,11 @@
       </c>
     </row>
     <row r="97">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C97" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1265,6 +1743,11 @@
       </c>
     </row>
     <row r="98">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 7 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C98" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1272,6 +1755,11 @@
       </c>
     </row>
     <row r="99">
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 8 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C99" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1279,6 +1767,11 @@
       </c>
     </row>
     <row r="100">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 9 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C100" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1286,6 +1779,11 @@
       </c>
     </row>
     <row r="101">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 10 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C101" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1293,6 +1791,11 @@
       </c>
     </row>
     <row r="102">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 11 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C102" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1300,6 +1803,11 @@
       </c>
     </row>
     <row r="103">
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 12 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C103" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -1307,6 +1815,11 @@
       </c>
     </row>
     <row r="104">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 13 ตำบลหูช้าง</t>
+        </is>
+      </c>
       <c r="C104" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -1319,6 +1832,11 @@
           <t>ตำบลห้วยแห้ง</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C105" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1326,6 +1844,11 @@
       </c>
     </row>
     <row r="106">
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C106" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1333,6 +1856,11 @@
       </c>
     </row>
     <row r="107">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C107" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1340,6 +1868,11 @@
       </c>
     </row>
     <row r="108">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C108" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1347,6 +1880,11 @@
       </c>
     </row>
     <row r="109">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 5 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C109" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1354,6 +1892,11 @@
       </c>
     </row>
     <row r="110">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 6 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C110" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1361,6 +1904,11 @@
       </c>
     </row>
     <row r="111">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 7 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C111" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1368,6 +1916,11 @@
       </c>
     </row>
     <row r="112">
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 8 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C112" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1375,6 +1928,11 @@
       </c>
     </row>
     <row r="113">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 9 ตำบลห้วยแห้ง</t>
+        </is>
+      </c>
       <c r="C113" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1387,6 +1945,11 @@
           <t>ตำบลเจ้าวัด</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C114" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1394,6 +1957,11 @@
       </c>
     </row>
     <row r="115">
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C115" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1401,6 +1969,11 @@
       </c>
     </row>
     <row r="116">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 3 ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C116" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1408,6 +1981,11 @@
       </c>
     </row>
     <row r="117">
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 4  ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C117" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1415,6 +1993,11 @@
       </c>
     </row>
     <row r="118">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 5 ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C118" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1422,6 +2005,11 @@
       </c>
     </row>
     <row r="119">
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 6 ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C119" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1429,6 +2017,11 @@
       </c>
     </row>
     <row r="120">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 7 ตำบลเจ้าวัด</t>
+        </is>
+      </c>
       <c r="C120" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1441,6 +2034,11 @@
           <t>ตำบลเมืองการุ้ง</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C121" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1448,6 +2046,11 @@
       </c>
     </row>
     <row r="122">
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 2 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C122" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1455,6 +2058,11 @@
       </c>
     </row>
     <row r="123">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 3 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C123" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1462,6 +2070,11 @@
       </c>
     </row>
     <row r="124">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>ศาลารวมใจศาลเจ้าแม่เมืองการุ้ง ม. 4 (นอกเขต+ในเขต)</t>
+        </is>
+      </c>
       <c r="C124" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1469,6 +2082,11 @@
       </c>
     </row>
     <row r="125">
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>วัดคลองโป่ง  หมู่ที่ 5 (นอกเขต+ในเขตเทศบาล)</t>
+        </is>
+      </c>
       <c r="C125" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1476,6 +2094,11 @@
       </c>
     </row>
     <row r="126">
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 6 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C126" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1483,6 +2106,11 @@
       </c>
     </row>
     <row r="127">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 7 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C127" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1490,6 +2118,11 @@
       </c>
     </row>
     <row r="128">
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 8 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C128" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1497,6 +2130,11 @@
       </c>
     </row>
     <row r="129">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 9 (นอกเขต+ในเขตเทศบาล)</t>
+        </is>
+      </c>
       <c r="C129" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1504,6 +2142,11 @@
       </c>
     </row>
     <row r="130">
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 10 ตำบลเมืองการุ้ง(นอกเขต+ในเขต)</t>
+        </is>
+      </c>
       <c r="C130" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1511,6 +2154,11 @@
       </c>
     </row>
     <row r="131">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน หมู่ที่ 11 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C131" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1518,6 +2166,11 @@
       </c>
     </row>
     <row r="132">
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 12 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C132" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -1525,6 +2178,11 @@
       </c>
     </row>
     <row r="133">
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน  หมู่ที่ 13 ตำบลเมืองการุ้ง</t>
+        </is>
+      </c>
       <c r="C133" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -1537,6 +2195,11 @@
           <t>ตำบลแก่นมะกรูด</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>ศาลากลางหมู่บ้าน   หมู่ที่ 1 ตำบลแก่นมะกรูด</t>
+        </is>
+      </c>
       <c r="C134" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1544,6 +2207,11 @@
       </c>
     </row>
     <row r="135">
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านคลองเสลา  หมู่ที่ 2 ตำบลแก่นมะกรูด</t>
+        </is>
+      </c>
       <c r="C135" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1551,6 +2219,11 @@
       </c>
     </row>
     <row r="136">
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านใหม่คลองอังวะ  หมู่ที่ 3 ตำบลแก่นมะกรูด</t>
+        </is>
+      </c>
       <c r="C136" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1558,6 +2231,11 @@
       </c>
     </row>
     <row r="137">
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านอีมาดอีทราย  หมู่ที่ 4 ตำบลแก่นมะกรูด</t>
+        </is>
+      </c>
       <c r="C137" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1606,6 +2284,11 @@
           <t>ตำบลทุ่งนางาม</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านดินแดง หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1613,6 +2296,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านห้วยโศก หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1620,6 +2308,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านชายเขา หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1627,6 +2320,11 @@
       </c>
     </row>
     <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านนิคมสามัคคี หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1634,6 +2332,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านการอดบ่วง หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1641,6 +2344,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหนองผักบุ้ง หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1648,6 +2356,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านน้ำวิ่ง หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1655,6 +2368,11 @@
       </c>
     </row>
     <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านทุ่งนางาม  หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1662,6 +2380,11 @@
       </c>
     </row>
     <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านบุ่งฝาง หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1669,6 +2392,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านศรีบุญเรือง หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1676,6 +2404,11 @@
       </c>
     </row>
     <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านประชาสุขสรรค์ หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1683,6 +2416,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมทุ่งเศรษฐี หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -1695,6 +2433,11 @@
           <t>ตำบลน้ำรอบ</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านน้ำรอบ หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1702,6 +2445,11 @@
       </c>
     </row>
     <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมหมู่บ้านห้วยทราย หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1709,6 +2457,11 @@
       </c>
     </row>
     <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านห้วยทราย หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1716,6 +2469,11 @@
       </c>
     </row>
     <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ศาลาการเปรียญวัดโป่งนวล หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1723,6 +2481,11 @@
       </c>
     </row>
     <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาผาแรต หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1730,6 +2493,11 @@
       </c>
     </row>
     <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านบุ่งกระเซอร์ หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1737,6 +2505,11 @@
       </c>
     </row>
     <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านบึงแห้ง หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1744,6 +2517,11 @@
       </c>
     </row>
     <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหนองเจ๊กกวย หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1751,6 +2529,11 @@
       </c>
     </row>
     <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านเนินมะค่า หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1758,6 +2541,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านโกรกลึก หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1765,6 +2553,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านซากุระพัฒนา หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1772,6 +2565,11 @@
       </c>
     </row>
     <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหนองม่วง หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -1779,6 +2577,11 @@
       </c>
     </row>
     <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านทรัพย์เจริญ หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -1786,6 +2589,11 @@
       </c>
     </row>
     <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านสวนใหม่ หมู่ที่ 13</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -1793,6 +2601,11 @@
       </c>
     </row>
     <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านห้วยน้ำดัง หมู่ที่ 14</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -1800,6 +2613,11 @@
       </c>
     </row>
     <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านทันสมัย หมู่ที่ 15</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>หน่วย 16</t>
@@ -1807,6 +2625,11 @@
       </c>
     </row>
     <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านผาสุขพัฒนา หมู่ที่ 16</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>หน่วย 17</t>
@@ -1814,6 +2637,11 @@
       </c>
     </row>
     <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านบึงแวง หมู่ที่ 17</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>หน่วย 18</t>
@@ -1821,6 +2649,11 @@
       </c>
     </row>
     <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านชินวัตรพัฒนา หมู่ที่ 19</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>หน่วย 19</t>
@@ -1833,6 +2666,11 @@
           <t>ตำบลประดู่ยืน</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านทัพยายปอน หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1840,6 +2678,11 @@
       </c>
     </row>
     <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านประดู่ยืน หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1847,6 +2690,11 @@
       </c>
     </row>
     <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหนองแขม หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1854,6 +2702,11 @@
       </c>
     </row>
     <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านตะคล้อ หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1861,6 +2714,11 @@
       </c>
     </row>
     <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านทุ่งสามแท่ง หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1868,6 +2726,11 @@
       </c>
     </row>
     <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหนองแหน หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1875,6 +2738,11 @@
       </c>
     </row>
     <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านหนองผักกาด หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1882,6 +2750,11 @@
       </c>
     </row>
     <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านใหม่ หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C40" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1889,6 +2762,11 @@
       </c>
     </row>
     <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านป่าคา หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C41" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1896,6 +2774,11 @@
       </c>
     </row>
     <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหนองปลาไหล หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C42" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1903,6 +2786,11 @@
       </c>
     </row>
     <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านวังหน้าศาล หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C43" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1910,6 +2798,11 @@
       </c>
     </row>
     <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านคลองโป่งพัฒนา หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C44" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -1922,6 +2815,11 @@
           <t>ตำบลป่าอ้อ</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์บ้านเขาฆ้องชัย หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -1929,6 +2827,11 @@
       </c>
     </row>
     <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ศาลาประชาคมบ้านเขาวง หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -1936,6 +2839,11 @@
       </c>
     </row>
     <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านคลองชะนี หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C47" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -1943,6 +2851,11 @@
       </c>
     </row>
     <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาน้ำโจน หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C48" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -1950,6 +2863,11 @@
       </c>
     </row>
     <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านป่าอ้อ หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C49" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -1957,6 +2875,11 @@
       </c>
     </row>
     <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านซับป่าพลู หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C50" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -1964,6 +2887,11 @@
       </c>
     </row>
     <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ศาลาการเปรียญวัดซับป่าพลู หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C51" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -1971,6 +2899,11 @@
       </c>
     </row>
     <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านคลองชะนี หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C52" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -1978,6 +2911,11 @@
       </c>
     </row>
     <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านซับป่าพลูใหม่ หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -1985,6 +2923,11 @@
       </c>
     </row>
     <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านป่าอ้อเหนือ หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -1992,6 +2935,11 @@
       </c>
     </row>
     <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาไม้นวน หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C55" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -1999,6 +2947,11 @@
       </c>
     </row>
     <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเนินม่วงพัฒนา หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C56" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -2011,6 +2964,11 @@
           <t>ตำบลระบำ</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ศาลาประชาคมบ้านท่ามะนาว หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C57" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2018,6 +2976,11 @@
       </c>
     </row>
     <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมหมู่บ้านห้วยรัง หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C58" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2025,6 +2988,11 @@
       </c>
     </row>
     <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านโป่งสามสิบ หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2032,6 +3000,11 @@
       </c>
     </row>
     <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านปางไม้ไผ่ หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2039,6 +3012,11 @@
       </c>
     </row>
     <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเพชรเจริญ หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C61" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2046,6 +3024,11 @@
       </c>
     </row>
     <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์ร้านค้าชุมชนบ้านเพชรเจริญ หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C62" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2053,6 +3036,11 @@
       </c>
     </row>
     <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านห้วยเปล้า หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C63" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2060,6 +3048,11 @@
       </c>
     </row>
     <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านโป่งมะค่า หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2067,6 +3060,11 @@
       </c>
     </row>
     <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านหาดทรายงาม หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C65" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2074,6 +3072,11 @@
       </c>
     </row>
     <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ศาลาประชาธิปไตยบ้านบึงเจริญ หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -2081,6 +3084,11 @@
       </c>
     </row>
     <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ศูนย์พัฒนาเด็กเล็กบ้านบึงเจริญ หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -2088,6 +3096,11 @@
       </c>
     </row>
     <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนห้วยขาแข้ง หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C68" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -2095,6 +3108,11 @@
       </c>
     </row>
     <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านอ่างห้วยดง หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C69" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -2102,6 +3120,11 @@
       </c>
     </row>
     <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านทรัพย์สมบูรณ์ หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C70" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -2109,6 +3132,11 @@
       </c>
     </row>
     <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านยางงาม หมู่ที่ 13</t>
+        </is>
+      </c>
       <c r="C71" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -2116,6 +3144,11 @@
       </c>
     </row>
     <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ศาลาประชาคมหมู่บ้านเขาเขียว หมู่ที่ 14</t>
+        </is>
+      </c>
       <c r="C72" t="inlineStr">
         <is>
           <t>หน่วย 16</t>
@@ -2123,6 +3156,11 @@
       </c>
     </row>
     <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านคีรีวงค์ หมู่ที่ 15</t>
+        </is>
+      </c>
       <c r="C73" t="inlineStr">
         <is>
           <t>หน่วย 17</t>
@@ -2130,6 +3168,11 @@
       </c>
     </row>
     <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาหินเทิน หมู่ที่ 16</t>
+        </is>
+      </c>
       <c r="C74" t="inlineStr">
         <is>
           <t>หน่วย 18</t>
@@ -2137,6 +3180,11 @@
       </c>
     </row>
     <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านพรเจริญ หมู่ที่ 17</t>
+        </is>
+      </c>
       <c r="C75" t="inlineStr">
         <is>
           <t>หน่วย 19</t>
@@ -2144,6 +3192,11 @@
       </c>
     </row>
     <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาไม้นวล หมู่ที่ 18</t>
+        </is>
+      </c>
       <c r="C76" t="inlineStr">
         <is>
           <t>หน่วย 20</t>
@@ -2151,6 +3204,11 @@
       </c>
     </row>
     <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านใหม่สามัคคี หมู่ที่ 19</t>
+        </is>
+      </c>
       <c r="C77" t="inlineStr">
         <is>
           <t>หน่วย 21</t>
@@ -2163,6 +3221,11 @@
           <t>ตำบลลานสัก</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านปากเหมือง หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C78" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2170,6 +3233,11 @@
       </c>
     </row>
     <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านพุหล่ม หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C79" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2177,6 +3245,11 @@
       </c>
     </row>
     <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ศาลาประชาคมบ้านเพชรน้ำผึ้ง หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C80" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2184,6 +3257,11 @@
       </c>
     </row>
     <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านเพชรน้ำผึ้ง หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C81" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2191,6 +3269,11 @@
       </c>
     </row>
     <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาดินเหนือ หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C82" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2198,6 +3281,11 @@
       </c>
     </row>
     <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ศาลาธรรมสังเวชวัดเขาดิน หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C83" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2205,6 +3293,11 @@
       </c>
     </row>
     <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านเขาพระยาพายเรือ หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C84" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2212,6 +3305,11 @@
       </c>
     </row>
     <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนเขาพระยาสังฆาราม หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C85" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2219,6 +3317,11 @@
       </c>
     </row>
     <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>อาคารอเนกประสงค์โรงเรียนบ้านร่องตาที หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C86" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2226,6 +3329,11 @@
       </c>
     </row>
     <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านร่องตาที หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C87" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -2233,6 +3341,11 @@
       </c>
     </row>
     <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านใหม่ไทยอีสาน หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -2240,6 +3353,11 @@
       </c>
     </row>
     <row r="89">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ศาลาการเปรียญวัดบ้านใหม่ไทยอีสาน หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C89" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -2247,6 +3365,11 @@
       </c>
     </row>
     <row r="90">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านสุขสวัสดิ์ หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C90" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -2254,6 +3377,11 @@
       </c>
     </row>
     <row r="91">
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านป่าสัก หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C91" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -2261,6 +3389,11 @@
       </c>
     </row>
     <row r="92">
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านสุขเสถียร หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C92" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -2268,6 +3401,11 @@
       </c>
     </row>
     <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ศาลาประชุม สปก. ช.4</t>
+        </is>
+      </c>
       <c r="C93" t="inlineStr">
         <is>
           <t>หน่วย 16</t>
@@ -2275,6 +3413,11 @@
       </c>
     </row>
     <row r="94">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ศาลาประชุมบ้านประสานสุข หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C94" t="inlineStr">
         <is>
           <t>หน่วย 17</t>
@@ -2282,6 +3425,11 @@
       </c>
     </row>
     <row r="95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ศูนย์ส่งเสริมการเรียนรู้อำเภอลานสัก (สกร.อ.ลานสัก) หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C95" t="inlineStr">
         <is>
           <t>หน่วย 18</t>
@@ -2289,6 +3437,11 @@
       </c>
     </row>
     <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ศาลากองทุนหมู่บ้าน หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C96" t="inlineStr">
         <is>
           <t>หน่วย 19</t>
@@ -2337,6 +3490,11 @@
           <t>ตำบลทุ่งโพ</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2344,6 +3502,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2351,6 +3514,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2358,6 +3526,11 @@
       </c>
     </row>
     <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2365,6 +3538,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2372,6 +3550,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ศาลาอเนกประสงค์  หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2379,6 +3562,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2386,6 +3574,11 @@
       </c>
     </row>
     <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2393,6 +3586,11 @@
       </c>
     </row>
     <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2400,6 +3598,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ศาลาอเนกประสงค์  หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -2407,6 +3610,11 @@
       </c>
     </row>
     <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -2414,6 +3622,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -2421,6 +3634,11 @@
       </c>
     </row>
     <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 13</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -2428,6 +3646,11 @@
       </c>
     </row>
     <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 14</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>หน่วย 14</t>
@@ -2435,6 +3658,11 @@
       </c>
     </row>
     <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน หมู่ที่ 15</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>หน่วย 15</t>
@@ -2447,6 +3675,11 @@
           <t>ตำบลเขากวางทอง</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>โรงเรียนทุ่งโพวิทยา  หมู่ที่ 1 ตำบลเขากวางทอง</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2454,6 +3687,11 @@
       </c>
     </row>
     <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2461,6 +3699,11 @@
       </c>
     </row>
     <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2468,6 +3711,11 @@
       </c>
     </row>
     <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2475,6 +3723,11 @@
       </c>
     </row>
     <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2482,6 +3735,11 @@
       </c>
     </row>
     <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านท่าชะอม  หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2489,6 +3747,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ศาลา SML  หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2496,6 +3759,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2503,6 +3771,11 @@
       </c>
     </row>
     <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2510,6 +3783,11 @@
       </c>
     </row>
     <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>หน่วย 10</t>
@@ -2517,6 +3795,11 @@
       </c>
     </row>
     <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 11</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>หน่วย 11</t>
@@ -2524,6 +3807,11 @@
       </c>
     </row>
     <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ศาลา SML  หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>หน่วย 12</t>
@@ -2531,6 +3819,11 @@
       </c>
     </row>
     <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน  หมู่ที่ 13</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>หน่วย 13</t>
@@ -2543,6 +3836,11 @@
           <t>ตำบลเขาบางแกรก</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ศาลาเฉลิมพระเกียรติ หมู่ที่ 1 (สระหลวง)</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2550,6 +3848,11 @@
       </c>
     </row>
     <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2557,6 +3860,11 @@
       </c>
     </row>
     <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2564,6 +3872,11 @@
       </c>
     </row>
     <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน หมู่ที่ 4 (ชุมชน 3)</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2571,6 +3884,11 @@
       </c>
     </row>
     <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ศาลาประชาคมเทศบาลตำบลเขาบางแกรก(ศาลเจ้าพ่อหลักเมือง)</t>
+        </is>
+      </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2578,6 +3896,11 @@
       </c>
     </row>
     <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน หมู่ที่ 4 (ชุมชน 8)</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2585,6 +3908,11 @@
       </c>
     </row>
     <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านทุ่งนาวิทยา</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2592,6 +3920,11 @@
       </c>
     </row>
     <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ศาลาอเนกประสงค์ หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2599,6 +3932,11 @@
       </c>
     </row>
     <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ศาลากลางบ้าน หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2647,6 +3985,11 @@
           <t>ตำบลทองหลาง</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านคลองแห้งวิทยา หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2654,6 +3997,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ศาลาการเปรียญวัดสมอทอง</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2661,6 +4009,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านละว้า หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2668,6 +4021,11 @@
       </c>
     </row>
     <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านตลิ่งสูง หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2675,6 +4033,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ศาลาเอนกประสงค์ อบต.ทองหลางหลังเก่า หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2682,6 +4045,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ศาลาการเปรียญวัดหนองผักแพว</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2689,6 +4057,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านป่าบัว หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2696,6 +4069,11 @@
       </c>
     </row>
     <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านคลองหวาย หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2703,6 +4081,11 @@
       </c>
     </row>
     <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านภูเหม็น หมู่ที่ 8</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2715,6 +4098,11 @@
           <t>ตำบลสุขฤทัย</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านวังบ่าง หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2722,6 +4110,11 @@
       </c>
     </row>
     <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้าน กกงิ้ว หมูที่ 2</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2729,6 +4122,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ศาลาการเปรียญวัดทุ่งสาลี</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2736,6 +4134,11 @@
       </c>
     </row>
     <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านหนองลัน หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2743,6 +4146,11 @@
       </c>
     </row>
     <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านหนองสี่เหลี่ยม หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2750,6 +4158,11 @@
       </c>
     </row>
     <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านชุมทอง หมู่ที่ 12</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2757,6 +4170,11 @@
       </c>
     </row>
     <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านหนองยาง หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2764,6 +4182,11 @@
       </c>
     </row>
     <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านล่องว่า หมู่ที่ 9</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2771,6 +4194,11 @@
       </c>
     </row>
     <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านวังบ่างสามัคคี หมู่ที่ 13</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>หน่วย 9</t>
@@ -2783,6 +4211,11 @@
           <t>ตำบลห้วยคต</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านชุมทหาร หมู่ที่ 1</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>หน่วย 1</t>
@@ -2790,6 +4223,11 @@
       </c>
     </row>
     <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>โรงเรียนอนุบาลห้วยคต หมู่ที่1</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>หน่วย 2</t>
@@ -2797,6 +4235,11 @@
       </c>
     </row>
     <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านหินโหง่น หมู่ที่ 2</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>หน่วย 3</t>
@@ -2804,6 +4247,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านป่าผาก หมู่ที่ 3</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>หน่วย 4</t>
@@ -2811,6 +4259,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>โรงเรียนบ้านกลาง หมู่ที่ 4</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>หน่วย 5</t>
@@ -2818,6 +4271,11 @@
       </c>
     </row>
     <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านหลังเขา หมู่ที่ 5</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>หน่วย 6</t>
@@ -2825,6 +4283,11 @@
       </c>
     </row>
     <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านบางกุ้ง หมู่ที่ 6</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>หน่วย 7</t>
@@ -2832,6 +4295,11 @@
       </c>
     </row>
     <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านหนองจอก หมู่ที่ 7</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>หน่วย 8</t>
@@ -2839,6 +4307,11 @@
       </c>
     </row>
     <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ศาลาประจำหมู่บ้านบ่อทราย หมู่ที่ 10</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>หน่วย 9</t>

</xml_diff>